<commit_message>
feat(store): deploy Pack 1 and Pack 2 landing pages, 58 wilayas order engine, and Vercel telemetry integration
</commit_message>
<xml_diff>
--- a/data/excel/Customers.xlsx
+++ b/data/excel/Customers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -627,9 +627,47 @@
         <v>2026-08-21T15:26:27.256Z</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>CUST-876147ff15e2</v>
+      </c>
+      <c r="B7" t="str">
+        <v>0555998877</v>
+      </c>
+      <c r="C7" t="str">
+        <v>عمر بن بلقاسم</v>
+      </c>
+      <c r="D7" t="str">
+        <v>1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>0</v>
+      </c>
+      <c r="F7" t="str">
+        <v>0</v>
+      </c>
+      <c r="G7" t="str">
+        <v>0</v>
+      </c>
+      <c r="H7" t="str">
+        <v>0</v>
+      </c>
+      <c r="I7" t="str">
+        <v>50</v>
+      </c>
+      <c r="J7" t="str">
+        <v>LOW</v>
+      </c>
+      <c r="K7" t="str">
+        <v>2026-10-05T17:49:22.783Z</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2026-10-05T17:49:23.010Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>